<commit_message>
docs(testing): add week 2 test cases TC011 to TC025
</commit_message>
<xml_diff>
--- a/HealthcareCRM/BugTracker.xlsx
+++ b/HealthcareCRM/BugTracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ff74d26e6023e292/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADF53F88-2AA5-47A7-B9A3-6DE47F214B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6463B2B2-416A-4E3D-847B-61D28C0246A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="138">
   <si>
     <t>Test #</t>
   </si>
@@ -194,6 +194,225 @@
     <t>Patient removed</t>
   </si>
   <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>Patient List</t>
+  </si>
+  <si>
+    <t>Page loads with all patients</t>
+  </si>
+  <si>
+    <t>Navigate to /Patient</t>
+  </si>
+  <si>
+    <t>Patient list displays with pagination</t>
+  </si>
+  <si>
+    <t>Patient list shown</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>Patient Search</t>
+  </si>
+  <si>
+    <t>Search by name</t>
+  </si>
+  <si>
+    <t>Type existing name in search bar</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>Search by phone</t>
+  </si>
+  <si>
+    <t>Type phone number in search bar</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>Search with no results</t>
+  </si>
+  <si>
+    <t>Type random text that doesnt exist</t>
+  </si>
+  <si>
+    <t>No patients found message shown</t>
+  </si>
+  <si>
+    <t>Empty state shown</t>
+  </si>
+  <si>
+    <t>TC015</t>
+  </si>
+  <si>
+    <t>Patient Detail</t>
+  </si>
+  <si>
+    <t>View patient details</t>
+  </si>
+  <si>
+    <t>Click Details button on any patient</t>
+  </si>
+  <si>
+    <t>Full patient profile shown</t>
+  </si>
+  <si>
+    <t>Profile displayed</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>Patient Create</t>
+  </si>
+  <si>
+    <t>Valid patient added</t>
+  </si>
+  <si>
+    <t>All fields filled correctly</t>
+  </si>
+  <si>
+    <t>Patient added</t>
+  </si>
+  <si>
+    <t>TC017</t>
+  </si>
+  <si>
+    <t>Empty form submission</t>
+  </si>
+  <si>
+    <t>All fields empty, click Save</t>
+  </si>
+  <si>
+    <t>Errors shown</t>
+  </si>
+  <si>
+    <t>TC018</t>
+  </si>
+  <si>
+    <t>Patient Edit</t>
+  </si>
+  <si>
+    <t>Update patient data</t>
+  </si>
+  <si>
+    <t>Change phone number, click Update</t>
+  </si>
+  <si>
+    <t>Updated data saved in list</t>
+  </si>
+  <si>
+    <t>Data updated</t>
+  </si>
+  <si>
+    <t>TC019</t>
+  </si>
+  <si>
+    <t>Patient Delete</t>
+  </si>
+  <si>
+    <t>Delete with confirmation</t>
+  </si>
+  <si>
+    <t>Click Delete, confirm in modal</t>
+  </si>
+  <si>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>Cancel delete</t>
+  </si>
+  <si>
+    <t>Click Delete, click Cancel in modal</t>
+  </si>
+  <si>
+    <t>Patient stays in list</t>
+  </si>
+  <si>
+    <t>Patient not deleted</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>Doctor List</t>
+  </si>
+  <si>
+    <t>Page loads</t>
+  </si>
+  <si>
+    <t>Navigate to /Doctor</t>
+  </si>
+  <si>
+    <t>Doctor list page shown</t>
+  </si>
+  <si>
+    <t>Page displayed</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>Doctor API</t>
+  </si>
+  <si>
+    <t>GET all doctors</t>
+  </si>
+  <si>
+    <t>Call GET /api/doctors</t>
+  </si>
+  <si>
+    <t>Returns active doctors list</t>
+  </si>
+  <si>
+    <t>JSON response returned</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>Empty state</t>
+  </si>
+  <si>
+    <t>No doctors in database</t>
+  </si>
+  <si>
+    <t>No doctors found message shown</t>
+  </si>
+  <si>
+    <t>Empty message shown</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>Response shape</t>
+  </si>
+  <si>
+    <t>Returns success, data, message shape</t>
+  </si>
+  <si>
+    <t>Correct shape returned</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t>Protected route</t>
+  </si>
+  <si>
+    <t>Access /Doctor without login</t>
+  </si>
+  <si>
+    <t>Redirected to login</t>
+  </si>
+  <si>
     <t>Bug #</t>
   </si>
   <si>
@@ -210,13 +429,19 @@
   </si>
   <si>
     <t>Fixed On</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  WEEK 2  PATIENT CRUD &amp; SEARCH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  WEEK 2  DOCTOR MODULE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -240,8 +465,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF375623"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,8 +504,28 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF595959"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF3FB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -293,11 +548,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -316,6 +586,25 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -619,15 +908,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
   </cols>
   <sheetData>
@@ -884,7 +1173,348 @@
         <v>12</v>
       </c>
     </row>
+    <row r="12" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+    </row>
+    <row r="13" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="G16" s="9"/>
+    </row>
+    <row r="17" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" s="9"/>
+    </row>
+    <row r="19" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="G22" s="9"/>
+    </row>
+    <row r="23" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+    </row>
+    <row r="24" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" s="9"/>
+    </row>
+    <row r="27" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="G28" s="9"/>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A23:G23"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -905,28 +1535,28 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>131</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>60</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>61</v>
+        <v>134</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>62</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
feat(week5): global error handler, loading states, network detection, 50+ test cases
</commit_message>
<xml_diff>
--- a/HealthcareCRM/BugTracker.xlsx
+++ b/HealthcareCRM/BugTracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ff74d26e6023e292/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADF53F88-2AA5-47A7-B9A3-6DE47F214B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6463B2B2-416A-4E3D-847B-61D28C0246A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="138">
   <si>
     <t>Test #</t>
   </si>
@@ -194,6 +194,225 @@
     <t>Patient removed</t>
   </si>
   <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>Patient List</t>
+  </si>
+  <si>
+    <t>Page loads with all patients</t>
+  </si>
+  <si>
+    <t>Navigate to /Patient</t>
+  </si>
+  <si>
+    <t>Patient list displays with pagination</t>
+  </si>
+  <si>
+    <t>Patient list shown</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>Patient Search</t>
+  </si>
+  <si>
+    <t>Search by name</t>
+  </si>
+  <si>
+    <t>Type existing name in search bar</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>Search by phone</t>
+  </si>
+  <si>
+    <t>Type phone number in search bar</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>Search with no results</t>
+  </si>
+  <si>
+    <t>Type random text that doesnt exist</t>
+  </si>
+  <si>
+    <t>No patients found message shown</t>
+  </si>
+  <si>
+    <t>Empty state shown</t>
+  </si>
+  <si>
+    <t>TC015</t>
+  </si>
+  <si>
+    <t>Patient Detail</t>
+  </si>
+  <si>
+    <t>View patient details</t>
+  </si>
+  <si>
+    <t>Click Details button on any patient</t>
+  </si>
+  <si>
+    <t>Full patient profile shown</t>
+  </si>
+  <si>
+    <t>Profile displayed</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>Patient Create</t>
+  </si>
+  <si>
+    <t>Valid patient added</t>
+  </si>
+  <si>
+    <t>All fields filled correctly</t>
+  </si>
+  <si>
+    <t>Patient added</t>
+  </si>
+  <si>
+    <t>TC017</t>
+  </si>
+  <si>
+    <t>Empty form submission</t>
+  </si>
+  <si>
+    <t>All fields empty, click Save</t>
+  </si>
+  <si>
+    <t>Errors shown</t>
+  </si>
+  <si>
+    <t>TC018</t>
+  </si>
+  <si>
+    <t>Patient Edit</t>
+  </si>
+  <si>
+    <t>Update patient data</t>
+  </si>
+  <si>
+    <t>Change phone number, click Update</t>
+  </si>
+  <si>
+    <t>Updated data saved in list</t>
+  </si>
+  <si>
+    <t>Data updated</t>
+  </si>
+  <si>
+    <t>TC019</t>
+  </si>
+  <si>
+    <t>Patient Delete</t>
+  </si>
+  <si>
+    <t>Delete with confirmation</t>
+  </si>
+  <si>
+    <t>Click Delete, confirm in modal</t>
+  </si>
+  <si>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>Cancel delete</t>
+  </si>
+  <si>
+    <t>Click Delete, click Cancel in modal</t>
+  </si>
+  <si>
+    <t>Patient stays in list</t>
+  </si>
+  <si>
+    <t>Patient not deleted</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>Doctor List</t>
+  </si>
+  <si>
+    <t>Page loads</t>
+  </si>
+  <si>
+    <t>Navigate to /Doctor</t>
+  </si>
+  <si>
+    <t>Doctor list page shown</t>
+  </si>
+  <si>
+    <t>Page displayed</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>Doctor API</t>
+  </si>
+  <si>
+    <t>GET all doctors</t>
+  </si>
+  <si>
+    <t>Call GET /api/doctors</t>
+  </si>
+  <si>
+    <t>Returns active doctors list</t>
+  </si>
+  <si>
+    <t>JSON response returned</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>Empty state</t>
+  </si>
+  <si>
+    <t>No doctors in database</t>
+  </si>
+  <si>
+    <t>No doctors found message shown</t>
+  </si>
+  <si>
+    <t>Empty message shown</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>Response shape</t>
+  </si>
+  <si>
+    <t>Returns success, data, message shape</t>
+  </si>
+  <si>
+    <t>Correct shape returned</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t>Protected route</t>
+  </si>
+  <si>
+    <t>Access /Doctor without login</t>
+  </si>
+  <si>
+    <t>Redirected to login</t>
+  </si>
+  <si>
     <t>Bug #</t>
   </si>
   <si>
@@ -210,13 +429,19 @@
   </si>
   <si>
     <t>Fixed On</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  WEEK 2  PATIENT CRUD &amp; SEARCH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  WEEK 2  DOCTOR MODULE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -240,8 +465,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF375623"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,8 +504,28 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF595959"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF3FB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -293,11 +548,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -316,6 +586,25 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -619,15 +908,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
   </cols>
   <sheetData>
@@ -884,7 +1173,348 @@
         <v>12</v>
       </c>
     </row>
+    <row r="12" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+    </row>
+    <row r="13" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="G16" s="9"/>
+    </row>
+    <row r="17" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" s="9"/>
+    </row>
+    <row r="19" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="G22" s="9"/>
+    </row>
+    <row r="23" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+    </row>
+    <row r="24" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="G24" s="9"/>
+    </row>
+    <row r="25" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="G25" s="9"/>
+    </row>
+    <row r="26" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" s="9"/>
+    </row>
+    <row r="27" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="G28" s="9"/>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A23:G23"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -905,28 +1535,28 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>131</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>59</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>60</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>61</v>
+        <v>134</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>62</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Add IsActive field and audit log support
</commit_message>
<xml_diff>
--- a/HealthcareCRM/BugTracker.xlsx
+++ b/HealthcareCRM/BugTracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ff74d26e6023e292/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6463B2B2-416A-4E3D-847B-61D28C0246A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADF53F88-2AA5-47A7-B9A3-6DE47F214B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="63">
   <si>
     <t>Test #</t>
   </si>
@@ -194,225 +194,6 @@
     <t>Patient removed</t>
   </si>
   <si>
-    <t>TC011</t>
-  </si>
-  <si>
-    <t>Patient List</t>
-  </si>
-  <si>
-    <t>Page loads with all patients</t>
-  </si>
-  <si>
-    <t>Navigate to /Patient</t>
-  </si>
-  <si>
-    <t>Patient list displays with pagination</t>
-  </si>
-  <si>
-    <t>Patient list shown</t>
-  </si>
-  <si>
-    <t>TC012</t>
-  </si>
-  <si>
-    <t>Patient Search</t>
-  </si>
-  <si>
-    <t>Search by name</t>
-  </si>
-  <si>
-    <t>Type existing name in search bar</t>
-  </si>
-  <si>
-    <t>TC013</t>
-  </si>
-  <si>
-    <t>Search by phone</t>
-  </si>
-  <si>
-    <t>Type phone number in search bar</t>
-  </si>
-  <si>
-    <t>TC014</t>
-  </si>
-  <si>
-    <t>Search with no results</t>
-  </si>
-  <si>
-    <t>Type random text that doesnt exist</t>
-  </si>
-  <si>
-    <t>No patients found message shown</t>
-  </si>
-  <si>
-    <t>Empty state shown</t>
-  </si>
-  <si>
-    <t>TC015</t>
-  </si>
-  <si>
-    <t>Patient Detail</t>
-  </si>
-  <si>
-    <t>View patient details</t>
-  </si>
-  <si>
-    <t>Click Details button on any patient</t>
-  </si>
-  <si>
-    <t>Full patient profile shown</t>
-  </si>
-  <si>
-    <t>Profile displayed</t>
-  </si>
-  <si>
-    <t>TC016</t>
-  </si>
-  <si>
-    <t>Patient Create</t>
-  </si>
-  <si>
-    <t>Valid patient added</t>
-  </si>
-  <si>
-    <t>All fields filled correctly</t>
-  </si>
-  <si>
-    <t>Patient added</t>
-  </si>
-  <si>
-    <t>TC017</t>
-  </si>
-  <si>
-    <t>Empty form submission</t>
-  </si>
-  <si>
-    <t>All fields empty, click Save</t>
-  </si>
-  <si>
-    <t>Errors shown</t>
-  </si>
-  <si>
-    <t>TC018</t>
-  </si>
-  <si>
-    <t>Patient Edit</t>
-  </si>
-  <si>
-    <t>Update patient data</t>
-  </si>
-  <si>
-    <t>Change phone number, click Update</t>
-  </si>
-  <si>
-    <t>Updated data saved in list</t>
-  </si>
-  <si>
-    <t>Data updated</t>
-  </si>
-  <si>
-    <t>TC019</t>
-  </si>
-  <si>
-    <t>Patient Delete</t>
-  </si>
-  <si>
-    <t>Delete with confirmation</t>
-  </si>
-  <si>
-    <t>Click Delete, confirm in modal</t>
-  </si>
-  <si>
-    <t>TC020</t>
-  </si>
-  <si>
-    <t>Cancel delete</t>
-  </si>
-  <si>
-    <t>Click Delete, click Cancel in modal</t>
-  </si>
-  <si>
-    <t>Patient stays in list</t>
-  </si>
-  <si>
-    <t>Patient not deleted</t>
-  </si>
-  <si>
-    <t>TC021</t>
-  </si>
-  <si>
-    <t>Doctor List</t>
-  </si>
-  <si>
-    <t>Page loads</t>
-  </si>
-  <si>
-    <t>Navigate to /Doctor</t>
-  </si>
-  <si>
-    <t>Doctor list page shown</t>
-  </si>
-  <si>
-    <t>Page displayed</t>
-  </si>
-  <si>
-    <t>TC022</t>
-  </si>
-  <si>
-    <t>Doctor API</t>
-  </si>
-  <si>
-    <t>GET all doctors</t>
-  </si>
-  <si>
-    <t>Call GET /api/doctors</t>
-  </si>
-  <si>
-    <t>Returns active doctors list</t>
-  </si>
-  <si>
-    <t>JSON response returned</t>
-  </si>
-  <si>
-    <t>TC023</t>
-  </si>
-  <si>
-    <t>Empty state</t>
-  </si>
-  <si>
-    <t>No doctors in database</t>
-  </si>
-  <si>
-    <t>No doctors found message shown</t>
-  </si>
-  <si>
-    <t>Empty message shown</t>
-  </si>
-  <si>
-    <t>TC024</t>
-  </si>
-  <si>
-    <t>Response shape</t>
-  </si>
-  <si>
-    <t>Returns success, data, message shape</t>
-  </si>
-  <si>
-    <t>Correct shape returned</t>
-  </si>
-  <si>
-    <t>TC025</t>
-  </si>
-  <si>
-    <t>Protected route</t>
-  </si>
-  <si>
-    <t>Access /Doctor without login</t>
-  </si>
-  <si>
-    <t>Redirected to login</t>
-  </si>
-  <si>
     <t>Bug #</t>
   </si>
   <si>
@@ -429,19 +210,13 @@
   </si>
   <si>
     <t>Fixed On</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  WEEK 2  PATIENT CRUD &amp; SEARCH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  WEEK 2  DOCTOR MODULE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -465,18 +240,8 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF375623"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,28 +269,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF595959"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEBF3FB"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -548,26 +293,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -586,25 +316,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -908,15 +619,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="38" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
-    <col min="6" max="6" width="28" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="10" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1173,348 +884,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-    </row>
-    <row r="13" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="G13" s="9"/>
-    </row>
-    <row r="14" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="G14" s="9"/>
-    </row>
-    <row r="15" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G15" s="9"/>
-    </row>
-    <row r="16" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="G16" s="9"/>
-    </row>
-    <row r="17" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="G17" s="9"/>
-    </row>
-    <row r="18" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="G18" s="9"/>
-    </row>
-    <row r="19" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G19" s="9"/>
-    </row>
-    <row r="20" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="G20" s="9"/>
-    </row>
-    <row r="21" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G21" s="9"/>
-    </row>
-    <row r="22" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="G22" s="9"/>
-    </row>
-    <row r="23" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-    </row>
-    <row r="24" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="G24" s="9"/>
-    </row>
-    <row r="25" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="G25" s="9"/>
-    </row>
-    <row r="26" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B26" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="F26" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="G26" s="9"/>
-    </row>
-    <row r="27" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="G27" s="9"/>
-    </row>
-    <row r="28" spans="1:7" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="E28" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="F28" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="G28" s="9"/>
-    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A23:G23"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1535,28 +905,28 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>131</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>132</v>
+        <v>59</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>133</v>
+        <v>60</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>134</v>
+        <v>61</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>135</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="25" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>